<commit_message>
Troca exemplos por cenários fictícios genéricos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XaeUyaSSWwJBaeSFHULPei
</commit_message>
<xml_diff>
--- a/planilha-80-20-chamados.xlsx
+++ b/planilha-80-20-chamados.xlsx
@@ -64,7 +64,7 @@
     <t xml:space="preserve">• Repita a análise no ciclo seguinte para confirmar se a correção realmente reduziu a fila.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Os dados de exemplo são ilustrativos: 140 chamados em 7 temas, em que 3 temas somam 80%.</t>
+    <t xml:space="preserve">• Os dados de exemplo são um cenário fictício: 140 chamados em 7 temas, em que 3 temas somam 80%. Apague-os antes de usar.</t>
   </si>
   <si>
     <t xml:space="preserve">Criado por Miller Barros · millerkbarros.github.io/portfolio-profissional</t>
@@ -106,22 +106,22 @@
     <t xml:space="preserve">Chave de ordenação</t>
   </si>
   <si>
-    <t xml:space="preserve">OS não sincroniza no mobile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baixa de material não grava</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Foto não anexa na OS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login expira em campo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relatório lento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Endereço incorreto</t>
+    <t xml:space="preserve">Falha de acesso / senha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erro ao emitir relatório</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lentidão no sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impressora</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E-mail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acesso a pastas</t>
   </si>
   <si>
     <t xml:space="preserve">Outros</t>
@@ -142,7 +142,7 @@
     <t xml:space="preserve">CH-1001</t>
   </si>
   <si>
-    <t xml:space="preserve">Exemplo ilustrativo</t>
+    <t xml:space="preserve">Cenário fictício</t>
   </si>
   <si>
     <t xml:space="preserve">CH-1002</t>
@@ -1041,22 +1041,22 @@
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>OS não sincroniza no mobile</c:v>
+                  <c:v>Falha de acesso / senha</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Baixa de material não grava</c:v>
+                  <c:v>Erro ao emitir relatório</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Foto não anexa na OS</c:v>
+                  <c:v>Lentidão no sistema</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Login expira em campo</c:v>
+                  <c:v>Impressora</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Relatório lento</c:v>
+                  <c:v>E-mail</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Endereço incorreto</c:v>
+                  <c:v>Acesso a pastas</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>Outros</c:v>
@@ -1106,8 +1106,8 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="23167149"/>
-        <c:axId val="77033600"/>
+        <c:axId val="7807812"/>
+        <c:axId val="30170067"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1171,22 +1171,22 @@
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>OS não sincroniza no mobile</c:v>
+                  <c:v>Falha de acesso / senha</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Baixa de material não grava</c:v>
+                  <c:v>Erro ao emitir relatório</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Foto não anexa na OS</c:v>
+                  <c:v>Lentidão no sistema</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Login expira em campo</c:v>
+                  <c:v>Impressora</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Relatório lento</c:v>
+                  <c:v>E-mail</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Endereço incorreto</c:v>
+                  <c:v>Acesso a pastas</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>Outros</c:v>
@@ -1243,11 +1243,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="49942818"/>
-        <c:axId val="40804039"/>
+        <c:axId val="26811170"/>
+        <c:axId val="5835561"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="23167149"/>
+        <c:axId val="7807812"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1279,7 +1279,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77033600"/>
+        <c:crossAx val="30170067"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1287,7 +1287,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="77033600"/>
+        <c:axId val="30170067"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1353,12 +1353,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23167149"/>
+        <c:crossAx val="7807812"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="49942818"/>
+        <c:axId val="26811170"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1390,7 +1390,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40804039"/>
+        <c:crossAx val="5835561"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1398,7 +1398,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40804039"/>
+        <c:axId val="5835561"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1466,7 +1466,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49942818"/>
+        <c:crossAx val="26811170"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1814,7 +1814,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="3" t="s">
         <v>13</v>
       </c>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="B5" s="10" t="str">
         <f aca="false">IF(LARGE(Temas!$C$2:$C$21,1)&lt;0,"",INDEX(Temas!$A$2:$A$21,MATCH(LARGE(Temas!$C$2:$C$21,1),Temas!$C$2:$C$21,0)))</f>
-        <v>OS não sincroniza no mobile</v>
+        <v>Falha de acesso / senha</v>
       </c>
       <c r="C5" s="10" t="n">
         <f aca="false">IF(B5="","",INDEX(Temas!$B$2:$B$21,MATCH(B5,Temas!$A$2:$A$21,0)))</f>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="B6" s="10" t="str">
         <f aca="false">IF(LARGE(Temas!$C$2:$C$21,2)&lt;0,"",INDEX(Temas!$A$2:$A$21,MATCH(LARGE(Temas!$C$2:$C$21,2),Temas!$C$2:$C$21,0)))</f>
-        <v>Baixa de material não grava</v>
+        <v>Erro ao emitir relatório</v>
       </c>
       <c r="C6" s="10" t="n">
         <f aca="false">IF(B6="","",INDEX(Temas!$B$2:$B$21,MATCH(B6,Temas!$A$2:$A$21,0)))</f>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="B7" s="10" t="str">
         <f aca="false">IF(LARGE(Temas!$C$2:$C$21,3)&lt;0,"",INDEX(Temas!$A$2:$A$21,MATCH(LARGE(Temas!$C$2:$C$21,3),Temas!$C$2:$C$21,0)))</f>
-        <v>Foto não anexa na OS</v>
+        <v>Lentidão no sistema</v>
       </c>
       <c r="C7" s="10" t="n">
         <f aca="false">IF(B7="","",INDEX(Temas!$B$2:$B$21,MATCH(B7,Temas!$A$2:$A$21,0)))</f>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B8" s="10" t="str">
         <f aca="false">IF(LARGE(Temas!$C$2:$C$21,4)&lt;0,"",INDEX(Temas!$A$2:$A$21,MATCH(LARGE(Temas!$C$2:$C$21,4),Temas!$C$2:$C$21,0)))</f>
-        <v>Login expira em campo</v>
+        <v>Impressora</v>
       </c>
       <c r="C8" s="10" t="n">
         <f aca="false">IF(B8="","",INDEX(Temas!$B$2:$B$21,MATCH(B8,Temas!$A$2:$A$21,0)))</f>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="B9" s="10" t="str">
         <f aca="false">IF(LARGE(Temas!$C$2:$C$21,5)&lt;0,"",INDEX(Temas!$A$2:$A$21,MATCH(LARGE(Temas!$C$2:$C$21,5),Temas!$C$2:$C$21,0)))</f>
-        <v>Relatório lento</v>
+        <v>E-mail</v>
       </c>
       <c r="C9" s="10" t="n">
         <f aca="false">IF(B9="","",INDEX(Temas!$B$2:$B$21,MATCH(B9,Temas!$A$2:$A$21,0)))</f>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="B10" s="10" t="str">
         <f aca="false">IF(LARGE(Temas!$C$2:$C$21,6)&lt;0,"",INDEX(Temas!$A$2:$A$21,MATCH(LARGE(Temas!$C$2:$C$21,6),Temas!$C$2:$C$21,0)))</f>
-        <v>Endereço incorreto</v>
+        <v>Acesso a pastas</v>
       </c>
       <c r="C10" s="10" t="n">
         <f aca="false">IF(B10="","",INDEX(Temas!$B$2:$B$21,MATCH(B10,Temas!$A$2:$A$21,0)))</f>

</xml_diff>